<commit_message>
adding job desc and recuiter params
</commit_message>
<xml_diff>
--- a/data/cv_render_new.xlsx
+++ b/data/cv_render_new.xlsx
@@ -447,17 +447,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Redesigned client segmentation model, improving customer behavior insights and targeting.</t>
+          <t>Led the redevelopment of the client segmentation model using Gaussian Mixture Modeling, applying feature engineering, hypothesis testing, and descriptive statistics to enhance clustering accuracy and business relevance.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Led A/B test design and analysis for home page, driving UX improvements.</t>
+          <t>Designed and analyzed A/B tests to optimize home page performance, maintaining key performance metric dashboards and supporting data-driven decision-making across teams.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Developed PySpark data pipeline to streamline accountancy data processing.</t>
+          <t>Developed scalable data pipelines with PySpark for processing and organizing large accountancy datasets, improving data accessibility and supporting supervised machine learning initiatives for targeted analyses.</t>
         </is>
       </c>
       <c r="L2" t="b">
@@ -492,17 +492,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Developed and deployed a 21-day promotional sales forecasting model using LGBM.</t>
+          <t>Led the development and deployment of a scalable, parallelized ML forecasting pipeline using Vertex AI and Kubeflow, reducing runtime from 6 hours to 40 minutes and enabling daily sales predictions for promotional events.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Optimized pipeline runtime from 6 hours to 40 minutes via code vectorization and parallelization.</t>
+          <t>Designed and implemented a rigorous experimental framework with hypothesis testing and causal inference to assess model impact on sales accuracy and inventory optimization, supporting risk analysis and continuous performance monitoring.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Implemented performance tracking and causal inference to validate model impact on sales.</t>
+          <t>Collaborated with stakeholders and data leadership to enhance transparency, explain statistical results, and guide strategic decisions using robust metrics like MAPE and wMAPE, improving adoption and model governance.</t>
         </is>
       </c>
       <c r="L3" t="b">
@@ -537,17 +537,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Developed daily country-level remittance volume forecasts, improving liquidity planning accuracy by ~10-12% MAPE.</t>
+          <t>Led the development of a production-grade forecasting system using LightGBM and ensemble methods to predict daily remittance volumes, improving liquidity planning and capital allocation across multiple markets.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Built and deployed AWS-based data pipeline and ML models using LightGBM, ensuring reliable daily predictions.</t>
+          <t>Designed and implemented robust, time-aware data pipelines and validation frameworks in AWS (S3, Athena), eliminating data leakage and ensuring temporal consistency for reliable model performance (~10–12% MAPE).</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Identified data leakage issues and enforced temporal consistency, enhancing model credibility and stakeholder trust.</t>
+          <t>Collaborated with senior stakeholders to translate business requirements into quantitative solutions, enhancing transparency, regulatory compliance, and decision-making around liquidity and operational risk.</t>
         </is>
       </c>
       <c r="L4" t="b">
@@ -637,22 +637,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>My area of expertise is tilted towards using statistics (Machine Learning included) to describe and understand client behavior, development of predictive models (e.g. churn or propension) and client segmentation using unsupervised ML. I have experience developing *ad hoc* analyses and also developing production ready models.</t>
+          <t>Developed predictive ML models for client behavior and segmentation</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Statistical modeling, data analysis and hypothesis testing are considered staple knowledge in the area I graduated from. This fact allowed me to transit between different technical areas seamlessly (such as machine learning, A/B testing and data visualization).</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>R is my language of choice, but I also have proficiency with Python, SQL and Spark (PySpark/Sparklyr). I work comfortably with git, github and Linux, besides also having experience working with the Data Bricks environment (and with notebooks in general) and AWS (e.g. Redshift and S3).</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>I have worked in several research projects with people from a wide array of backgrounds and seniority levels, some of which from end-to-end. I have been well trained since an undergrad to explain technical subjects to non technical audiences.</t>
+          <t>Proficient in Python, SQL, R, Spark, and cloud environments (AWS, Databricks)</t>
         </is>
       </c>
       <c r="L7" t="b">

</xml_diff>

<commit_message>
adding skills stack function and updating
</commit_message>
<xml_diff>
--- a/data/cv_render_new.xlsx
+++ b/data/cv_render_new.xlsx
@@ -354,7 +354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -447,22 +447,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Redesigned client segmentation model using Gaussian Mixture Modeling, applying feature engineering and hypothesis testing to validate new variables.</t>
+          <t>Redesigned client segmentation using Gaussian Mixture Modeling, applying feature engineering, hypothesis testing, and descriptive statistics for model refinement.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Designed and analyzed A/B tests for home page redesign, improving experimental robustness and guiding stakeholder decisions with clear insights.</t>
+          <t>Led home page redesign experiments, executing A/B testing and reducing click-through rate time by 20%.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Developed PySpark data pipelines to process and structure complex accountancy data, enhancing data accessibility and accuracy for financial reporting.</t>
+          <t>Developed PySpark data pipelines for efficient processing and analysis of accounting data from multiple sources.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Mentored junior analysts in statistical methods, experimentation, and machine learning deployment, fostering team analytical capabilities and best practices.</t>
+          <t>Designed and analyzed randomized experiments to assess customer behavior and model performance metrics.</t>
         </is>
       </c>
       <c r="L2" t="b">
@@ -497,22 +497,22 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Developed and deployed ML forecasting model predicting promotional sales 21 days ahead, achieving 20% MAPE for FMCG product demand.</t>
+          <t>Developed and deployed a machine learning forecasting model predicting FMCG promotional event sales 21 days ahead with 20% MAPE accuracy.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Led creation of ETL pipeline integrating product sales data for supply teams, enabling informed inventory decision-making and forecasting accuracy.</t>
+          <t>Led creation of automated ETL pipelines integrating sales data into supply team workflows, enhancing data accessibility and orchestration.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Collaborated with MLOps to deploy daily parallelized sales prediction pipeline using Vertex AI and Kubeflow, reducing process time from 6 hours to 40 minutes.</t>
+          <t>Collaborated with ML Operations to deploy daily parallelized sales predictions using Vertex AI and Kubeflow, reducing runtime from 6 hours to 40 minutes.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Implemented experimental design with causal inference, measuring model impact through hypothesis testing against baseline sales and stock surplus averages.</t>
+          <t>Created causal inference experiments and hypothesis testing frameworks to measure model impact, validating $4 million monthly overstock cost savings.</t>
         </is>
       </c>
       <c r="L3" t="b">
@@ -547,22 +547,22 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Developed and deployed forecasting models predicting daily remittance volumes at a country level with 10–15% MAPE across markets.</t>
+          <t>Developed and deployed an ML forecasting system achieving 10% MAPE accuracy, surpassing manual remittance volume predictions across multiple countries.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Designed robust data pipelines using AWS S3 and Athena to ensure reliable, consistent datasets for model development and validation.</t>
+          <t>Saved approximately $500,000 daily by reducing underfunding via accurate daily liquidity forecasts for a pilot country.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Implemented tree-based ML models with LightGBM ensembles, combining strong experimentation to achieve stable, realistic forecasts.</t>
+          <t>Reduced lockout rates by 25%, decreasing customer disruptions caused by correspondent agents' underfunding through predictive modeling.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Identified and eliminated data leakage by restructuring feature engineering pipelines with strict temporal validation frameworks.</t>
+          <t>Cut remittance prediction processing time from 3 hours to 7 minutes, automating workflows and reducing headcount needs significantly.</t>
         </is>
       </c>
       <c r="L4" t="b">
@@ -636,36 +636,6 @@
         </is>
       </c>
       <c r="L6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>academic_articles</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Skills &amp; stack</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Specialized in statistical modeling and machine learning to analyze client behavior, develop churn and propensity models, and perform client segmentation using unsupervised techniques.</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Skilled in building predictive models and creating production-ready solutions using R, Python, SQL, and Spark (PySpark/Sparklyr).</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Proficient in hypothesis testing, data visualization, and A/B testing to extract insights and validate data-driven experiments.</t>
-        </is>
-      </c>
-      <c r="L7" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adding prompt logic and parameters
</commit_message>
<xml_diff>
--- a/data/cv_render_new.xlsx
+++ b/data/cv_render_new.xlsx
@@ -354,7 +354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -447,22 +447,22 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Redesigned client segmentation using Gaussian Mixture Modeling, applying feature engineering, hypothesis testing, and descriptive statistics for model refinement.</t>
+          <t>Redesigned and validated client segmentation model using Gaussian Mixture Modeling, descriptive statistics, and hypothesis testing for improved clustering quality.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Led home page redesign experiments, executing A/B testing and reducing click-through rate time by 20%.</t>
+          <t>Analyzed A/B test results and designed experiments to optimize homepage user engagement, reducing click-through rate time by 20%.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Developed PySpark data pipelines for efficient processing and analysis of accounting data from multiple sources.</t>
+          <t>Developed a Pyspark data pipeline to efficiently process and scrutinize financial accountancy data, enhancing data accessibility and reliability.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Designed and analyzed randomized experiments to assess customer behavior and model performance metrics.</t>
+          <t>Built and maintained key performance dashboards using Python, SQL, and Databricks, supporting real-time monitoring of experimentation metrics.</t>
         </is>
       </c>
       <c r="L2" t="b">
@@ -497,22 +497,22 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Developed and deployed a machine learning forecasting model predicting FMCG promotional event sales 21 days ahead with 20% MAPE accuracy.</t>
+          <t>Developed and deployed a forecasting model predicting promotional FMCG sales 21 days ahead, achieving 20% MAPE accuracy.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Led creation of automated ETL pipelines integrating sales data into supply team workflows, enhancing data accessibility and orchestration.</t>
+          <t>Designed an ETL pipeline and ML workflow that prevented overstock, generating $4 million monthly savings while maintaining sales levels.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Collaborated with ML Operations to deploy daily parallelized sales predictions using Vertex AI and Kubeflow, reducing runtime from 6 hours to 40 minutes.</t>
+          <t>Collaborated with MLOps to deploy parallelized sales prediction pipelines on Vertex AI and Kubeflow, reducing runtime from 6 hours to 40 minutes.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Created causal inference experiments and hypothesis testing frameworks to measure model impact, validating $4 million monthly overstock cost savings.</t>
+          <t>Built a model performance database to monitor KPIs, track bugs, and communicate statistical robustness and forecast reliability to stakeholders.</t>
         </is>
       </c>
       <c r="L3" t="b">
@@ -547,22 +547,22 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Developed and deployed an ML forecasting system achieving 10% MAPE accuracy, surpassing manual remittance volume predictions across multiple countries.</t>
+          <t>Developed and deployed ML forecasting models predicting daily remittance volumes at country level with 10% MAPE accuracy.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Saved approximately $500,000 daily by reducing underfunding via accurate daily liquidity forecasts for a pilot country.</t>
+          <t>Streamlined data pipelines using AWS S3, Athena, and containerized environments to ensure reliable, scalable production predictions.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Reduced lockout rates by 25%, decreasing customer disruptions caused by correspondent agents' underfunding through predictive modeling.</t>
+          <t>Saved approximately $500,000 daily by reducing underfunding in pilot country through automated, data-driven liquidity planning models.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Cut remittance prediction processing time from 3 hours to 7 minutes, automating workflows and reducing headcount needs significantly.</t>
+          <t>Reduced correspondent agent lockout rates by 25% via improved prediction models, increasing transaction success and customer satisfaction.</t>
         </is>
       </c>
       <c r="L4" t="b">
@@ -636,6 +636,36 @@
         </is>
       </c>
       <c r="L6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>skills_stack</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Skills &amp; stack</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Statistical modeling, causal inference, price elasticity, marketing mix modelling expertise</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Python, SQL, cloud platforms (AWS, GCP), ML deployment, MLOps tools (Kubeflow, Docker, CI/CD)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Data visualization (Power BI, Looker), stakeholder communication, FMCG domain knowledge, mentoring</t>
+        </is>
+      </c>
+      <c r="L7" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added expertise logic and bash config run
</commit_message>
<xml_diff>
--- a/data/cv_render_new.xlsx
+++ b/data/cv_render_new.xlsx
@@ -447,17 +447,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Developed a K-prototypes clustering model for client segmentation, enabling targeted marketing campaigns that increased coupon conversion rates by 20%.</t>
+          <t>Developed an unsupervised K-prototypes clustering model to segment clients using demographic and behavioral data, enabling targeted marketing campaigns.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Created a real-time client activity monitoring pipeline, “activity status,” to identify engagement stages and reduce overall churn through timely interventions.</t>
+          <t>Created a real-time client activity monitoring pipeline to identify engagement stages, reducing churn and improving campaign response rates.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Reformulated churn metrics with statistical rigor, improving measurement accuracy and supporting data-driven retention strategies across client segments.</t>
+          <t>Redesigned churn metrics with statistically robust methods to better capture client behavior and retention patterns across the platform.</t>
         </is>
       </c>
       <c r="L2" t="b">
@@ -492,17 +492,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Developed and deployed a 21-day promotional sales forecasting model using LGBM, achieving 20% MAPE for FMCG demand predictions.</t>
+          <t>Designed and deployed a 21-day sales forecasting model for FMCG promotional events, achieving 20% MAPE accuracy across stores.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Created an orchestrated ETL pipeline integrating product sales data for supply teams, enabling daily parallel training for store-specific models.</t>
+          <t>Led development of an orchestrated ETL pipeline to provide clean, real-time product sales data to supply teams using SQL and Python.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Collaborated with MLOps to deploy pipelines with Vertex AI and Kubeflow, reducing process runtime from 6 hours to 40 minutes through code optimization.</t>
+          <t>Collaborated with MLOps to deploy parallelized daily sales prediction pipelines using Vertex AI and Kubeflow, reducing runtime from 6 hours to 40 minutes.</t>
         </is>
       </c>
       <c r="L3" t="b">
@@ -537,17 +537,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Developed a production-grade forecasting system predicting daily remittance volumes with 10% MAPE accuracy, outperforming manual processes.</t>
+          <t>Developed a forecasting model predicting daily remittance volumes with 10% MAPE, outperforming manual processes across multiple countries.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Engineered data pipelines using AWS S3 and Athena, ensuring consistent, reliable datasets for modeling and validation workflows.</t>
+          <t>Built robust data pipelines integrating AWS S3 and Athena, enabling consistent, reliable data for accurate real-time liquidity modeling.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Designed and validated tree-based ML models with LightGBM, implementing robust time-aware validation to prevent data leakage.</t>
+          <t>Achieved daily savings of approximately $500,000 by reducing underfunding risks, driving significant capital allocation efficiency improvements.</t>
         </is>
       </c>
       <c r="L4" t="b">
@@ -637,22 +637,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>LookML for semantic modeling and building scalable BI dashboards.</t>
+          <t>Defined KPIs and developed business analytics frameworks driving actionable insights.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Databricks dashboards for real-time data visualization and KPI monitoring.</t>
+          <t>Built interactive dashboards using LookML and Looker for real-time decision support.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Looker dashboards to deliver actionable business insights across teams.</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Quarto and R Markdown for reproducible reporting and dynamic documentation.</t>
+          <t>Designed and maintained Databricks dashboards with Quarto and R Markdown for reporting.</t>
         </is>
       </c>
       <c r="L7" t="b">
@@ -672,22 +667,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Google Cloud Platform: Vertex AI, BigQuery, and GCS for scalable ML workflows and data storage</t>
+          <t>Owned end-to-end batch ML pipelines on GCP and AWS using Vertex AI, Kubeflow, BigQuery, and Athena.</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>AWS ecosystem: S3, Athena, ECS Fargate, ECR, Glue, and EventBridge for data lakes and orchestration</t>
+          <t>Implemented model monitoring, versioning, and CI/CD workflows with GitHub Actions and containerized ECS/Fargate deployments.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Kubeflow pipelines for batch ML pipelines, model monitoring, tracking, and deployment automation</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>CI/CD with GitHub Actions and Terraform IaC for reproducible, production-grade ML system delivery</t>
+          <t>Orchestrated large-scale data processing and vectorization, optimizing performance across S3, Glue, EventBridge, and Terraform infrastructure.</t>
         </is>
       </c>
       <c r="L8" t="b">
@@ -707,22 +697,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>LightGBM and logistic regression for classification and regression tasks with rigorous model evaluation.</t>
+          <t>Applied logistic regression, LightGBM, and tree-based models for robust predictive modeling.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Custom feature engineering for time series forecasting using temporal validation and backtesting techniques.</t>
+          <t>Engineered custom features for time series forecasting with rigorous temporal validation and backtesting.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Clustering with k-prototypes for customer segmentation and data-driven grouping strategies.</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Model performance metrics including MAPE, AUC, Average Precision, and lift for robust evaluation.</t>
+          <t>Designed clustering solutions using k-prototypes for market segmentation, optimizing model evaluation metrics.</t>
         </is>
       </c>
       <c r="L9" t="b">
@@ -742,22 +727,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Python, pandas, NumPy, scikit-learn, LightGBM for model training, evaluation, and production pipelines</t>
+          <t>Built production ML pipelines using Python, Pandas, NumPy, Scikit-learn, and LightGBM for robust market modeling.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SQL and awswrangler for analytical querying, data modeling, and interaction with cloud data warehouses</t>
+          <t>Deployed reproducible, modular ML systems with Docker, Git versioning, and automated Bash scripting on Linux environments.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>PySpark and Databricks for distributed data processing and scalable machine learning workflows</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Docker containerization, Git, and modular Python packaging for reproducible ML environments and CI/CD integration</t>
+          <t>Managed data workflows and analytics using SQL, PySpark, Databricks, and awswrangler with UUID-based tracking and packaging.</t>
         </is>
       </c>
       <c r="L10" t="b">
@@ -777,22 +757,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Applied Bayesian inference and maximum likelihood for probabilistic model evaluation and refinement.</t>
+          <t>Designed and analyzed experiments using hypothesis testing and rigorous experimental frameworks</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Utilized bootstrapping and resampling techniques in Python to estimate model performance variability.</t>
+          <t>Applied bootstrapping and resampling methods for robust statistical validation and uncertainty estimation</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Designed experiments and hypothesis tests to validate ML model impacts using statistical frameworks.</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Analyzed summary and rolling metrics for continuous monitoring of model behavior over time.</t>
+          <t>Implemented Bayesian inference and maximum likelihood techniques for advanced probabilistic modeling</t>
         </is>
       </c>
       <c r="L11" t="b">

</xml_diff>